<commit_message>
Changes of reporting manager
</commit_message>
<xml_diff>
--- a/public/sample/users_import.xlsx
+++ b/public/sample/users_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{455BB341-DB38-4F75-AAC4-E416689D631C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26279EDA-5799-4B99-88E2-BEDE4F25C067}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -91,7 +91,7 @@
     <t>Department</t>
   </si>
   <si>
-    <t>reporting_manager_id</t>
+    <t>ReportingManager</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Changes of user sample
</commit_message>
<xml_diff>
--- a/public/sample/users_import.xlsx
+++ b/public/sample/users_import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26279EDA-5799-4B99-88E2-BEDE4F25C067}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A126696C-5129-4D25-AED2-632279F07CDB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,40 @@
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Pc</author>
+  </authors>
+  <commentList>
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{A6C37592-917F-45B5-91D1-A99E2E7460F1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Pc:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Please enter employee id of the reporting manager</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -98,7 +132,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -110,6 +144,19 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -350,7 +397,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -4520,5 +4567,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>